<commit_message>
fix: renderActivity closing brace + ev.labelKey notif bug; feat(A): multi-hotel uses kpis_hoteles.xlsx Calipolis data (3 hotels, real metrics), improved KPI cards CSS vars; feat(A): AR Real better UX (balance alert, clearer button); feat(A): multi-hotel table improved with color-coded metrics
</commit_message>
<xml_diff>
--- a/datos-referencia/reservas_credito.xlsx
+++ b/datos-referencia/reservas_credito.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="65">
   <si>
     <t>numero_reserva</t>
   </si>
@@ -109,6 +109,78 @@
     <t>Iberdrola Clientes SAU</t>
   </si>
   <si>
+    <t>2027-04-06</t>
+  </si>
+  <si>
+    <t>2027-04-11</t>
+  </si>
+  <si>
+    <t>2027-03-17</t>
+  </si>
+  <si>
+    <t>2027-04-21</t>
+  </si>
+  <si>
+    <t>2027-03-07</t>
+  </si>
+  <si>
+    <t>2027-02-20</t>
+  </si>
+  <si>
+    <t>2027-04-16</t>
+  </si>
+  <si>
+    <t>2027-03-27</t>
+  </si>
+  <si>
+    <t>2027-02-10</t>
+  </si>
+  <si>
+    <t>2027-04-26</t>
+  </si>
+  <si>
+    <t>2027-01-31</t>
+  </si>
+  <si>
+    <t>2027-01-21</t>
+  </si>
+  <si>
+    <t>2027-04-09</t>
+  </si>
+  <si>
+    <t>2027-04-13</t>
+  </si>
+  <si>
+    <t>2027-03-20</t>
+  </si>
+  <si>
+    <t>2027-04-23</t>
+  </si>
+  <si>
+    <t>2027-03-10</t>
+  </si>
+  <si>
+    <t>2027-02-25</t>
+  </si>
+  <si>
+    <t>2027-04-18</t>
+  </si>
+  <si>
+    <t>2027-03-29</t>
+  </si>
+  <si>
+    <t>2027-02-13</t>
+  </si>
+  <si>
+    <t>2027-04-28</t>
+  </si>
+  <si>
+    <t>2027-02-02</t>
+  </si>
+  <si>
+    <t>2027-01-24</t>
+  </si>
+  <si>
     <t>PENDIENTE_FACTURA</t>
   </si>
   <si>
@@ -116,25 +188,35 @@
   </si>
   <si>
     <t>COBRADO</t>
+  </si>
+  <si>
+    <t>2027-03-22</t>
+  </si>
+  <si>
+    <t>2027-03-12</t>
+  </si>
+  <si>
+    <t>2027-02-27</t>
+  </si>
+  <si>
+    <t>2027-04-01</t>
+  </si>
+  <si>
+    <t>2027-02-15</t>
+  </si>
+  <si>
+    <t>2027-02-05</t>
+  </si>
+  <si>
+    <t>2027-01-26</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
-  </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -150,7 +232,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -158,31 +240,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -481,37 +544,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -522,11 +585,11 @@
       <c r="B2" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="2">
-        <v>46148</v>
-      </c>
-      <c r="D2" s="2">
-        <v>46151</v>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
+        <v>43</v>
       </c>
       <c r="E2">
         <v>4</v>
@@ -544,7 +607,7 @@
         <v>3200</v>
       </c>
       <c r="J2" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -554,11 +617,11 @@
       <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="2">
-        <v>46153</v>
-      </c>
-      <c r="D3" s="2">
-        <v>46155</v>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>44</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -576,7 +639,7 @@
         <v>1600</v>
       </c>
       <c r="J3" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -586,11 +649,11 @@
       <c r="B4" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="2">
-        <v>46128</v>
-      </c>
-      <c r="D4" s="2">
-        <v>46131</v>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>45</v>
       </c>
       <c r="E4">
         <v>8</v>
@@ -608,10 +671,10 @@
         <v>6720</v>
       </c>
       <c r="J4" t="s">
-        <v>32</v>
-      </c>
-      <c r="K4" s="2">
-        <v>46133</v>
+        <v>56</v>
+      </c>
+      <c r="K4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -621,11 +684,11 @@
       <c r="B5" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="2">
-        <v>46163</v>
-      </c>
-      <c r="D5" s="2">
-        <v>46165</v>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>46</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -643,7 +706,7 @@
         <v>2370</v>
       </c>
       <c r="J5" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -653,11 +716,11 @@
       <c r="B6" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="2">
-        <v>46118</v>
-      </c>
-      <c r="D6" s="2">
-        <v>46121</v>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>47</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -675,10 +738,10 @@
         <v>4000</v>
       </c>
       <c r="J6" t="s">
-        <v>32</v>
-      </c>
-      <c r="K6" s="2">
-        <v>46123</v>
+        <v>56</v>
+      </c>
+      <c r="K6" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -688,11 +751,11 @@
       <c r="B7" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="2">
-        <v>46103</v>
-      </c>
-      <c r="D7" s="2">
-        <v>46108</v>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" t="s">
+        <v>48</v>
       </c>
       <c r="E7">
         <v>12</v>
@@ -710,10 +773,10 @@
         <v>10600</v>
       </c>
       <c r="J7" t="s">
-        <v>32</v>
-      </c>
-      <c r="K7" s="2">
-        <v>46110</v>
+        <v>56</v>
+      </c>
+      <c r="K7" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -723,11 +786,11 @@
       <c r="B8" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="2">
-        <v>46158</v>
-      </c>
-      <c r="D8" s="2">
-        <v>46160</v>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" t="s">
+        <v>49</v>
       </c>
       <c r="E8">
         <v>2</v>
@@ -745,7 +808,7 @@
         <v>1480</v>
       </c>
       <c r="J8" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -755,11 +818,11 @@
       <c r="B9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="2">
-        <v>46138</v>
-      </c>
-      <c r="D9" s="2">
-        <v>46140</v>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>50</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -777,10 +840,10 @@
         <v>1480</v>
       </c>
       <c r="J9" t="s">
-        <v>32</v>
-      </c>
-      <c r="K9" s="2">
-        <v>46143</v>
+        <v>56</v>
+      </c>
+      <c r="K9" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -790,11 +853,11 @@
       <c r="B10" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="2">
-        <v>46093</v>
-      </c>
-      <c r="D10" s="2">
-        <v>46096</v>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>51</v>
       </c>
       <c r="E10">
         <v>6</v>
@@ -812,10 +875,10 @@
         <v>4850</v>
       </c>
       <c r="J10" t="s">
-        <v>32</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46098</v>
+        <v>56</v>
+      </c>
+      <c r="K10" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -825,11 +888,11 @@
       <c r="B11" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="2">
-        <v>46168</v>
-      </c>
-      <c r="D11" s="2">
-        <v>46170</v>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>52</v>
       </c>
       <c r="E11">
         <v>6</v>
@@ -847,7 +910,7 @@
         <v>4950</v>
       </c>
       <c r="J11" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -857,11 +920,11 @@
       <c r="B12" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="2">
-        <v>46083</v>
-      </c>
-      <c r="D12" s="2">
-        <v>46085</v>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>53</v>
       </c>
       <c r="E12">
         <v>3</v>
@@ -879,10 +942,10 @@
         <v>2300</v>
       </c>
       <c r="J12" t="s">
-        <v>33</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46088</v>
+        <v>57</v>
+      </c>
+      <c r="K12" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -892,11 +955,11 @@
       <c r="B13" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="2">
-        <v>46073</v>
-      </c>
-      <c r="D13" s="2">
-        <v>46076</v>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" t="s">
+        <v>54</v>
       </c>
       <c r="E13">
         <v>4</v>
@@ -914,10 +977,10 @@
         <v>3150</v>
       </c>
       <c r="J13" t="s">
-        <v>33</v>
-      </c>
-      <c r="K13" s="2">
-        <v>46078</v>
+        <v>57</v>
+      </c>
+      <c r="K13" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>